<commit_message>
made some changes to etsting excel
</commit_message>
<xml_diff>
--- a/testing.xlsx
+++ b/testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/roryschram/Documents/Work/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B2BBB20-1E09-C149-991D-96606B1AA031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB0A2BB-E863-5F4F-B24C-39A3F1B2E73E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16640" xr2:uid="{B2F224B3-2683-8A46-B4CF-646FB0916998}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16640" activeTab="1" xr2:uid="{B2F224B3-2683-8A46-B4CF-646FB0916998}"/>
   </bookViews>
   <sheets>
     <sheet name="USRP Power" sheetId="4" r:id="rId1"/>
@@ -18,17 +18,7 @@
     <sheet name="Range Testing" sheetId="2" r:id="rId3"/>
     <sheet name="Classification Testing" sheetId="3" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.4" hidden="1">'USRP Power'!$D$3</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'USRP Power'!$D$4:$D$21</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'USRP Power'!$G$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'USRP Power'!$G$4:$G$21</definedName>
-    <definedName name="_xlchart.v2.0" hidden="1">'USRP Power'!$D$3</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">'USRP Power'!$D$4:$D$21</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">'USRP Power'!$G$3</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">'USRP Power'!$G$4:$G$21</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,15 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>Small Loopback</t>
-  </si>
-  <si>
-    <t>Transmit Gain</t>
-  </si>
-  <si>
-    <t>Receive Gain</t>
   </si>
   <si>
     <t>Attenuation</t>
@@ -83,12 +67,51 @@
   <si>
     <t>received_dBFS</t>
   </si>
+  <si>
+    <t>snr_dB_1</t>
+  </si>
+  <si>
+    <t>BER_1</t>
+  </si>
+  <si>
+    <t>snr_dB_2</t>
+  </si>
+  <si>
+    <t>BER_2</t>
+  </si>
+  <si>
+    <t>snr_dB_3</t>
+  </si>
+  <si>
+    <t>BER_3</t>
+  </si>
+  <si>
+    <t>snr_dB_4</t>
+  </si>
+  <si>
+    <t>BER_4</t>
+  </si>
+  <si>
+    <t>snr_dB_5</t>
+  </si>
+  <si>
+    <t>BER_5</t>
+  </si>
+  <si>
+    <t>avg_snr_dB</t>
+  </si>
+  <si>
+    <t>avg_BER</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -101,6 +124,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -497,7 +526,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1629,24 +1658,24 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
         <v>6</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1921,10 +1950,10 @@
     </row>
     <row r="25" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D25" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.2">
@@ -1944,7 +1973,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200B8DD6-86B7-2D45-9650-9EE6C1C0ADA5}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -1953,23 +1982,601 @@
     <col min="4" max="4" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>1.4790000000000001</v>
+      </c>
+      <c r="D3">
+        <v>49.767000000000003</v>
+      </c>
+      <c r="E3">
+        <v>1.4710000000000001</v>
+      </c>
+      <c r="F3">
+        <v>49.744999999999997</v>
+      </c>
+      <c r="G3">
+        <v>1.504</v>
+      </c>
+      <c r="H3">
+        <v>49.57</v>
+      </c>
+      <c r="I3">
+        <v>1.478</v>
+      </c>
+      <c r="J3">
+        <v>49.796999999999997</v>
+      </c>
+      <c r="K3">
+        <v>1.355</v>
+      </c>
+      <c r="L3">
+        <v>49.24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>99</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B30">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B31">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B32">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B34">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B36">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B37">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B38">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B39">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B40">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B41">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B42">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B43">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B44">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B45">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B46">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B47">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B48">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B49">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B50">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B52">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B53">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B54">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B55">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B56">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B57">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B58">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B59">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B60">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B61">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B62">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B63">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B64">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B65">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B66">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B67">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B68">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B69">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B70">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B71">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B72">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B73">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B74">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B75">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B76">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B77">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B78">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B79">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B80">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B81">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B82">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B83">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B84">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B85">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B86">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B87">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B88">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B89">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B90">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B91">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B92">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B93">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B94">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B95">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B96">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B97">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B98">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B99">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B100">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B101">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B103">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>